<commit_message>
refresh generated PNAD metadata
</commit_message>
<xml_diff>
--- a/data/metadata/df_metadata.xlsx
+++ b/data/metadata/df_metadata.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q51"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,25 +479,30 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>income_scale_divisor</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Exchange</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Index</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Adjust2025</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Inflation</t>
         </is>
@@ -538,21 +543,24 @@
       <c r="L2" t="n">
         <v>9999999</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>11.313</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>100</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>4.6292535</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>5.6292535</v>
       </c>
     </row>
@@ -591,21 +599,24 @@
       <c r="L3" t="n">
         <v>999999999</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>14.93</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>106.42361</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>4.28947805848721</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>5.28947805848721</v>
       </c>
     </row>
@@ -644,21 +655,24 @@
       <c r="L4" t="n">
         <v>999999999</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>19.05</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>115.45139</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>3.875864638788671</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>4.875864638788671</v>
       </c>
     </row>
@@ -697,21 +711,24 @@
       <c r="L5" t="n">
         <v>999999999</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>28.792</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>129.16667</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>3.358131629467571</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>4.358131629467571</v>
       </c>
     </row>
@@ -732,15 +749,18 @@
         <v>0</v>
       </c>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -785,21 +805,24 @@
       <c r="L7" t="n">
         <v>9999999</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>105.284</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>161.63194</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>2.482760585562482</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>3.482760585562482</v>
       </c>
     </row>
@@ -838,21 +861,24 @@
       <c r="L8" t="n">
         <v>9999999</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>202.088</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>169.61806</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>2.318781915086164</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>3.318781915086164</v>
       </c>
     </row>
@@ -903,21 +929,24 @@
       <c r="L9" t="n">
         <v>9999999</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>701.381</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>174.30556</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>2.229531806099587</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>3.229531806099587</v>
       </c>
     </row>
@@ -964,21 +993,24 @@
       <c r="L10" t="n">
         <v>9999999</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>2203.947</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>181.77083</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>2.096895965100671</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>3.096895965100671</v>
       </c>
     </row>
@@ -1025,21 +1057,24 @@
       <c r="L11" t="n">
         <v>999999999</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>7461.667</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>187.67361</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>1.999491244400318</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>2.999491244400318</v>
       </c>
     </row>
@@ -1086,21 +1121,24 @@
       <c r="L12" t="n">
         <v>999999999</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="inlineStr">
         <is>
           <t>cruzado-Cz$</t>
         </is>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>13.84</v>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>190.97222</v>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>1.947681867027571</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>2.947681867027571</v>
       </c>
     </row>
@@ -1147,21 +1185,24 @@
       <c r="L13" t="n">
         <v>999999999</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" t="inlineStr">
         <is>
           <t>cruzado-Cz$</t>
         </is>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>49.866</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>199.13194</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>1.826896328132996</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>2.826896328132996</v>
       </c>
     </row>
@@ -1212,21 +1253,24 @@
       <c r="L14" t="n">
         <v>999999999</v>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" t="inlineStr">
         <is>
           <t>cruzado-Cz$</t>
         </is>
       </c>
-      <c r="N14" t="n">
+      <c r="O14" t="n">
         <v>326.235</v>
       </c>
-      <c r="O14" t="n">
+      <c r="P14" t="n">
         <v>207.46528</v>
       </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
         <v>1.71334726466038</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="R14" t="n">
         <v>2.71334726466038</v>
       </c>
     </row>
@@ -1273,21 +1317,24 @@
       <c r="L15" t="n">
         <v>999999999</v>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="inlineStr">
         <is>
           <t>cruzado novo-NCz$</t>
         </is>
       </c>
-      <c r="N15" t="n">
+      <c r="O15" t="n">
         <v>3.267</v>
       </c>
-      <c r="O15" t="n">
+      <c r="P15" t="n">
         <v>216.66667</v>
       </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
         <v>1.59811696002897</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="R15" t="n">
         <v>2.59811696002897</v>
       </c>
     </row>
@@ -1334,21 +1381,24 @@
       <c r="L16" t="n">
         <v>999999999</v>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>75.541</v>
       </c>
-      <c r="O16" t="n">
+      <c r="P16" t="n">
         <v>230.03472</v>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>1.447132111187389</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="R16" t="n">
         <v>2.447132111187389</v>
       </c>
     </row>
@@ -1369,15 +1419,18 @@
         <v>0</v>
       </c>
       <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
+      <c r="M17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1422,21 +1475,24 @@
       <c r="L18" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M18" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" t="inlineStr">
         <is>
           <t>cruzeiro-Cr$</t>
         </is>
       </c>
-      <c r="N18" t="n">
+      <c r="O18" t="n">
         <v>5771.524</v>
       </c>
-      <c r="O18" t="n">
+      <c r="P18" t="n">
         <v>244.96528</v>
       </c>
-      <c r="P18" t="n">
+      <c r="Q18" t="n">
         <v>1.297980146410953</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="R18" t="n">
         <v>2.297980146410953</v>
       </c>
     </row>
@@ -1483,21 +1539,24 @@
       <c r="L19" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" t="inlineStr">
         <is>
           <t>cruzeiro real-CR$</t>
         </is>
       </c>
-      <c r="N19" t="n">
+      <c r="O19" t="n">
         <v>111.189</v>
       </c>
-      <c r="O19" t="n">
+      <c r="P19" t="n">
         <v>251.73611</v>
       </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
         <v>1.236172434697588</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="R19" t="n">
         <v>2.236172434697588</v>
       </c>
     </row>
@@ -1518,15 +1577,18 @@
         <v>0</v>
       </c>
       <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr">
+      <c r="M20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1571,21 +1633,24 @@
       <c r="L21" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M21" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N21" t="n">
+      <c r="O21" t="n">
         <v>0.9528</v>
       </c>
-      <c r="O21" t="n">
+      <c r="P21" t="n">
         <v>265.79861</v>
       </c>
-      <c r="P21" t="n">
+      <c r="Q21" t="n">
         <v>1.117864160388198</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="R21" t="n">
         <v>2.117864160388198</v>
       </c>
     </row>
@@ -1632,21 +1697,24 @@
       <c r="L22" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="M22" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N22" t="n">
+      <c r="O22" t="n">
         <v>1.0193</v>
       </c>
-      <c r="O22" t="n">
+      <c r="P22" t="n">
         <v>273.78472</v>
       </c>
-      <c r="P22" t="n">
+      <c r="Q22" t="n">
         <v>1.056087534760888</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="R22" t="n">
         <v>2.056087534760888</v>
       </c>
     </row>
@@ -1693,21 +1761,24 @@
       <c r="L23" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M23" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N23" t="n">
+      <c r="O23" t="n">
         <v>1.0936</v>
       </c>
-      <c r="O23" t="n">
+      <c r="P23" t="n">
         <v>279.86111</v>
       </c>
-      <c r="P23" t="n">
+      <c r="Q23" t="n">
         <v>1.011445427340726</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="R23" t="n">
         <v>2.011445427340726</v>
       </c>
     </row>
@@ -1754,21 +1825,24 @@
       <c r="L24" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M24" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N24" t="n">
+      <c r="O24" t="n">
         <v>1.1809</v>
       </c>
-      <c r="O24" t="n">
+      <c r="P24" t="n">
         <v>283.85417</v>
       </c>
-      <c r="P24" t="n">
+      <c r="Q24" t="n">
         <v>0.9831498335923687</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="R24" t="n">
         <v>1.983149833592369</v>
       </c>
     </row>
@@ -1815,21 +1889,24 @@
       <c r="L25" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="M25" t="n">
+        <v>1</v>
+      </c>
+      <c r="N25" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N25" t="n">
+      <c r="O25" t="n">
         <v>1.8981</v>
       </c>
-      <c r="O25" t="n">
+      <c r="P25" t="n">
         <v>291.31944</v>
       </c>
-      <c r="P25" t="n">
+      <c r="Q25" t="n">
         <v>0.9323301939616526</v>
       </c>
-      <c r="Q25" t="n">
+      <c r="R25" t="n">
         <v>1.932330193961653</v>
       </c>
     </row>
@@ -1850,15 +1927,18 @@
         <v>0</v>
       </c>
       <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr">
+      <c r="M26" t="n">
+        <v>1</v>
+      </c>
+      <c r="N26" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1903,21 +1983,24 @@
       <c r="L27" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="M27" t="n">
+        <v>1</v>
+      </c>
+      <c r="N27" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N27" t="n">
+      <c r="O27" t="n">
         <v>2.6717</v>
       </c>
-      <c r="O27" t="n">
+      <c r="P27" t="n">
         <v>309.20139</v>
       </c>
-      <c r="P27" t="n">
+      <c r="Q27" t="n">
         <v>0.820578329224199</v>
       </c>
-      <c r="Q27" t="n">
+      <c r="R27" t="n">
         <v>1.820578329224199</v>
       </c>
     </row>
@@ -1964,21 +2047,24 @@
       <c r="L28" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M28" t="n">
+        <v>1</v>
+      </c>
+      <c r="N28" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N28" t="n">
+      <c r="O28" t="n">
         <v>3.342</v>
       </c>
-      <c r="O28" t="n">
+      <c r="P28" t="n">
         <v>313.88889</v>
       </c>
-      <c r="P28" t="n">
+      <c r="Q28" t="n">
         <v>0.7933904892269363</v>
       </c>
-      <c r="Q28" t="n">
+      <c r="R28" t="n">
         <v>1.793390489226936</v>
       </c>
     </row>
@@ -2025,21 +2111,24 @@
       <c r="L29" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M29" t="n">
+        <v>1</v>
+      </c>
+      <c r="N29" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N29" t="n">
+      <c r="O29" t="n">
         <v>2.9228</v>
       </c>
-      <c r="O29" t="n">
+      <c r="P29" t="n">
         <v>321.35417</v>
       </c>
-      <c r="P29" t="n">
+      <c r="Q29" t="n">
         <v>0.7517287857195067</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="R29" t="n">
         <v>1.751728785719507</v>
       </c>
     </row>
@@ -2078,21 +2167,24 @@
       <c r="L30" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="M30" t="n">
+        <v>1</v>
+      </c>
+      <c r="N30" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N30" t="n">
+      <c r="O30" t="n">
         <v>2.8911</v>
       </c>
-      <c r="O30" t="n">
+      <c r="P30" t="n">
         <v>329.51389</v>
       </c>
-      <c r="P30" t="n">
+      <c r="Q30" t="n">
         <v>0.70835089834908</v>
       </c>
-      <c r="Q30" t="n">
+      <c r="R30" t="n">
         <v>1.70835089834908</v>
       </c>
     </row>
@@ -2131,21 +2223,24 @@
       <c r="L31" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="M31" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N31" t="n">
+      <c r="O31" t="n">
         <v>2.2944</v>
       </c>
-      <c r="O31" t="n">
+      <c r="P31" t="n">
         <v>345.13889</v>
       </c>
-      <c r="P31" t="n">
+      <c r="Q31" t="n">
         <v>0.6310110691959401</v>
       </c>
-      <c r="Q31" t="n">
+      <c r="R31" t="n">
         <v>1.63101106919594</v>
       </c>
     </row>
@@ -2184,21 +2279,24 @@
       <c r="L32" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M32" t="n">
+        <v>1</v>
+      </c>
+      <c r="N32" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N32" t="n">
+      <c r="O32" t="n">
         <v>2.1687</v>
       </c>
-      <c r="O32" t="n">
+      <c r="P32" t="n">
         <v>352.08333</v>
       </c>
-      <c r="P32" t="n">
+      <c r="Q32" t="n">
         <v>0.5988412459061894</v>
       </c>
-      <c r="Q32" t="n">
+      <c r="R32" t="n">
         <v>1.598841245906189</v>
       </c>
     </row>
@@ -2237,21 +2335,24 @@
       <c r="L33" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M33" t="n">
+        <v>1</v>
+      </c>
+      <c r="N33" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N33" t="n">
+      <c r="O33" t="n">
         <v>1.8996</v>
       </c>
-      <c r="O33" t="n">
+      <c r="P33" t="n">
         <v>362.06076</v>
       </c>
-      <c r="P33" t="n">
+      <c r="Q33" t="n">
         <v>0.5547814405515803</v>
       </c>
-      <c r="Q33" t="n">
+      <c r="R33" t="n">
         <v>1.55478144055158</v>
       </c>
     </row>
@@ -2290,21 +2391,24 @@
       <c r="L34" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M34" t="n">
+        <v>1</v>
+      </c>
+      <c r="N34" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N34" t="n">
+      <c r="O34" t="n">
         <v>1.7996</v>
       </c>
-      <c r="O34" t="n">
+      <c r="P34" t="n">
         <v>379.99479</v>
       </c>
-      <c r="P34" t="n">
+      <c r="Q34" t="n">
         <v>0.4814028108122217</v>
       </c>
-      <c r="Q34" t="n">
+      <c r="R34" t="n">
         <v>1.481402810812222</v>
       </c>
     </row>
@@ -2343,21 +2447,24 @@
       <c r="L35" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="M35" t="n">
+        <v>1</v>
+      </c>
+      <c r="N35" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N35" t="n">
+      <c r="O35" t="n">
         <v>1.8198</v>
       </c>
-      <c r="O35" t="n">
+      <c r="P35" t="n">
         <v>374.75868</v>
       </c>
-      <c r="P35" t="n">
+      <c r="Q35" t="n">
         <v>0.5021008986369573</v>
       </c>
-      <c r="Q35" t="n">
+      <c r="R35" t="n">
         <v>1.502100898636957</v>
       </c>
     </row>
@@ -2378,15 +2485,18 @@
         <v>0</v>
       </c>
       <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr">
+      <c r="M36" t="n">
+        <v>1</v>
+      </c>
+      <c r="N36" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2423,21 +2533,24 @@
       <c r="L37" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="M37" t="n">
+        <v>1</v>
+      </c>
+      <c r="N37" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N37" t="n">
+      <c r="O37" t="n">
         <v>1.7498</v>
       </c>
-      <c r="O37" t="n">
+      <c r="P37" t="n">
         <v>393.39757</v>
       </c>
-      <c r="P37" t="n">
+      <c r="Q37" t="n">
         <v>0.4309324533956831</v>
       </c>
-      <c r="Q37" t="n">
+      <c r="R37" t="n">
         <v>1.430932453395683</v>
       </c>
     </row>
@@ -2476,21 +2589,24 @@
       <c r="L38" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="M38" t="n">
+        <v>1</v>
+      </c>
+      <c r="N38" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N38" t="n">
+      <c r="O38" t="n">
         <v>2.0281</v>
       </c>
-      <c r="O38" t="n">
+      <c r="P38" t="n">
         <v>401.06771</v>
       </c>
-      <c r="P38" t="n">
+      <c r="Q38" t="n">
         <v>0.4035668690456282</v>
       </c>
-      <c r="Q38" t="n">
+      <c r="R38" t="n">
         <v>1.403566869045628</v>
       </c>
     </row>
@@ -2529,21 +2645,24 @@
       <c r="L39" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="M39" t="n">
+        <v>1</v>
+      </c>
+      <c r="N39" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N39" t="n">
+      <c r="O39" t="n">
         <v>2.2705</v>
       </c>
-      <c r="O39" t="n">
+      <c r="P39" t="n">
         <v>405.45833</v>
       </c>
-      <c r="P39" t="n">
+      <c r="Q39" t="n">
         <v>0.3883679489332479</v>
       </c>
-      <c r="Q39" t="n">
+      <c r="R39" t="n">
         <v>1.388367948933248</v>
       </c>
     </row>
@@ -2582,21 +2701,24 @@
       <c r="L40" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="M40" t="n">
+        <v>1</v>
+      </c>
+      <c r="N40" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N40" t="n">
+      <c r="O40" t="n">
         <v>2.3329</v>
       </c>
-      <c r="O40" t="n">
+      <c r="P40" t="n">
         <v>412.28646</v>
       </c>
-      <c r="P40" t="n">
+      <c r="Q40" t="n">
         <v>0.3653743322058163</v>
       </c>
-      <c r="Q40" t="n">
+      <c r="R40" t="n">
         <v>1.365374332205816</v>
       </c>
     </row>
@@ -2635,21 +2757,24 @@
       <c r="L41" t="n">
         <v>999999999999</v>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="M41" t="n">
+        <v>1</v>
+      </c>
+      <c r="N41" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N41" t="n">
+      <c r="O41" t="n">
         <v>3.9065</v>
       </c>
-      <c r="O41" t="n">
+      <c r="P41" t="n">
         <v>412.32292</v>
       </c>
-      <c r="P41" t="n">
+      <c r="Q41" t="n">
         <v>0.3652535978354052</v>
       </c>
-      <c r="Q41" t="n">
+      <c r="R41" t="n">
         <v>1.365253597835405</v>
       </c>
     </row>
@@ -2688,21 +2813,24 @@
       <c r="L42" t="n">
         <v>999999</v>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M42" t="n">
+        <v>1</v>
+      </c>
+      <c r="N42" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N42" t="n">
+      <c r="O42" t="n">
         <v>3.2564</v>
       </c>
-      <c r="O42" t="n">
+      <c r="P42" t="n">
         <v>418.70833</v>
       </c>
-      <c r="P42" t="n">
+      <c r="Q42" t="n">
         <v>0.3444331284261768</v>
       </c>
-      <c r="Q42" t="n">
+      <c r="R42" t="n">
         <v>1.344433128426177</v>
       </c>
     </row>
@@ -2741,21 +2869,24 @@
       <c r="L43" t="n">
         <v>999999</v>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="M43" t="n">
+        <v>100</v>
+      </c>
+      <c r="N43" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N43" t="n">
+      <c r="O43" t="n">
         <v>3.1348</v>
       </c>
-      <c r="O43" t="n">
+      <c r="P43" t="n">
         <v>427.83854</v>
       </c>
-      <c r="P43" t="n">
+      <c r="Q43" t="n">
         <v>0.3157424994952533</v>
       </c>
-      <c r="Q43" t="n">
+      <c r="R43" t="n">
         <v>1.315742499495253</v>
       </c>
     </row>
@@ -2794,21 +2925,24 @@
       <c r="L44" t="n">
         <v>999999</v>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="M44" t="n">
+        <v>1</v>
+      </c>
+      <c r="N44" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N44" t="n">
+      <c r="O44" t="n">
         <v>4.1165</v>
       </c>
-      <c r="O44" t="n">
+      <c r="P44" t="n">
         <v>437.81597</v>
       </c>
-      <c r="P44" t="n">
+      <c r="Q44" t="n">
         <v>0.28575791787586</v>
       </c>
-      <c r="Q44" t="n">
+      <c r="R44" t="n">
         <v>1.28575791787586</v>
       </c>
     </row>
@@ -2847,21 +2981,24 @@
       <c r="L45" t="n">
         <v>999999</v>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="M45" t="n">
+        <v>1</v>
+      </c>
+      <c r="N45" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N45" t="n">
+      <c r="O45" t="n">
         <v>4.1215</v>
       </c>
-      <c r="O45" t="n">
+      <c r="P45" t="n">
         <v>445.19097</v>
       </c>
-      <c r="P45" t="n">
+      <c r="Q45" t="n">
         <v>0.2644581492746809</v>
       </c>
-      <c r="Q45" t="n">
+      <c r="R45" t="n">
         <v>1.264458149274681</v>
       </c>
     </row>
@@ -2900,21 +3037,24 @@
       <c r="L46" t="n">
         <v>999999</v>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="M46" t="n">
+        <v>1</v>
+      </c>
+      <c r="N46" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N46" t="n">
+      <c r="O46" t="n">
         <v>5.3995</v>
       </c>
-      <c r="O46" t="n">
+      <c r="P46" t="n">
         <v>451.38368</v>
       </c>
-      <c r="P46" t="n">
+      <c r="Q46" t="n">
         <v>0.2471105512720353</v>
       </c>
-      <c r="Q46" t="n">
+      <c r="R46" t="n">
         <v>1.247110551272035</v>
       </c>
     </row>
@@ -2953,21 +3093,24 @@
       <c r="L47" t="n">
         <v>999999</v>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="M47" t="n">
+        <v>1</v>
+      </c>
+      <c r="N47" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N47" t="n">
+      <c r="O47" t="n">
         <v>5.2797</v>
       </c>
-      <c r="O47" t="n">
+      <c r="P47" t="n">
         <v>475.53819</v>
       </c>
-      <c r="P47" t="n">
+      <c r="Q47" t="n">
         <v>0.1837647571481063</v>
       </c>
-      <c r="Q47" t="n">
+      <c r="R47" t="n">
         <v>1.183764757148106</v>
       </c>
     </row>
@@ -3006,21 +3149,24 @@
       <c r="L48" t="n">
         <v>999999</v>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="M48" t="n">
+        <v>1</v>
+      </c>
+      <c r="N48" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N48" t="n">
+      <c r="O48" t="n">
         <v>5.237</v>
       </c>
-      <c r="O48" t="n">
+      <c r="P48" t="n">
         <v>514.49479</v>
       </c>
-      <c r="P48" t="n">
+      <c r="Q48" t="n">
         <v>0.09413226516832185</v>
       </c>
-      <c r="Q48" t="n">
+      <c r="R48" t="n">
         <v>1.094132265168322</v>
       </c>
     </row>
@@ -3059,21 +3205,24 @@
       <c r="L49" t="n">
         <v>999999</v>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="M49" t="n">
+        <v>1</v>
+      </c>
+      <c r="N49" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N49" t="n">
+      <c r="O49" t="n">
         <v>4.937</v>
       </c>
-      <c r="O49" t="n">
+      <c r="P49" t="n">
         <v>533.46528</v>
       </c>
-      <c r="P49" t="n">
+      <c r="Q49" t="n">
         <v>0.05522396884010883</v>
       </c>
-      <c r="Q49" t="n">
+      <c r="R49" t="n">
         <v>1.055223968840109</v>
       </c>
     </row>
@@ -3112,21 +3261,24 @@
       <c r="L50" t="n">
         <v>999999</v>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="M50" t="n">
+        <v>1</v>
+      </c>
+      <c r="N50" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N50" t="n">
+      <c r="O50" t="n">
         <v>5.5416</v>
       </c>
-      <c r="O50" t="n">
+      <c r="P50" t="n">
         <v>546.40972</v>
       </c>
-      <c r="P50" t="n">
+      <c r="Q50" t="n">
         <v>0.03022572512070254</v>
       </c>
-      <c r="Q50" t="n">
+      <c r="R50" t="n">
         <v>1.030225725120703</v>
       </c>
     </row>
@@ -3165,21 +3317,24 @@
       <c r="L51" t="n">
         <v>999999</v>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="M51" t="n">
+        <v>1</v>
+      </c>
+      <c r="N51" t="inlineStr">
         <is>
           <t>Real R$</t>
         </is>
       </c>
-      <c r="N51" t="n">
+      <c r="O51" t="n">
         <v>5.3674</v>
       </c>
-      <c r="O51" t="n">
+      <c r="P51" t="n">
         <v>562.92535</v>
       </c>
-      <c r="P51" t="n">
+      <c r="Q51" t="n">
         <v>0</v>
       </c>
-      <c r="Q51" t="n">
+      <c r="R51" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>